<commit_message>
feat: update server port to 8000 and adjust frontend API proxy settings
- Changed server port from 8080 to 8000 in application.yml and updated Vite config for API proxy.
- Modified the Excel import functionality to handle Spanish date formats and added tests for date validation.
- Introduced a new PortfolioValuationIntegrationTest to validate portfolio calculations and summaries.
- Enhanced the dashboard with improved error handling, performance metrics, and detailed position reporting.
- Updated Spanish translations for dashboard and import functionalities.
- Added new styles for portfolio alerts and position sections in the frontend.
</commit_message>
<xml_diff>
--- a/backend/src/main/resources/templates/plantilla_importacion_portafolio.xlsx
+++ b/backend/src/main/resources/templates/plantilla_importacion_portafolio.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" r:id="R41e2e01683914d36"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operaciones" sheetId="2" r:id="Re6075de76944414d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ejemplos" sheetId="3" r:id="Rac4d62b64c204c5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" r:id="R7d13d46f69f6410e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operaciones" sheetId="2" r:id="R27f5f7a0d23a4d25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ejemplos" sheetId="3" r:id="R439bd10899aa427f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,10 +15,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="3">
+  <x:numFmts count="4">
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
     <x:numFmt numFmtId="201" formatCode="#,##0.########"/>
     <x:numFmt numFmtId="202" formatCode="#,##0.00"/>
+    <x:numFmt numFmtId="203" formatCode="dd/mm/yyyy"/>
   </x:numFmts>
   <x:fonts count="12">
     <x:font>
@@ -286,7 +287,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="149">
+  <x:cellXfs count="155">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -625,6 +626,24 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="11" fillId="5" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="9" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="9" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="9" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -993,7 +1012,7 @@
         <x:v>Sí</x:v>
       </x:c>
       <x:c r="C13" s="44" t="str">
-        <x:v>yyyy-mm-dd</x:v>
+        <x:v>dd/mm/aaaa o aaaa-mm-dd</x:v>
       </x:c>
       <x:c r="D13" s="44" t="str">
         <x:v>Fecha real de la operación. No puede ser futura.</x:v>
@@ -1253,7 +1272,7 @@
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="92"/>
+      <x:c r="A2" s="149"/>
       <x:c r="B2" s="89"/>
       <x:c r="C2" s="89"/>
       <x:c r="D2" s="89"/>
@@ -1266,7 +1285,7 @@
       <x:c r="I2" s="101"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="93"/>
+      <x:c r="A3" s="150"/>
       <x:c r="B3" s="90"/>
       <x:c r="C3" s="90"/>
       <x:c r="D3" s="90"/>
@@ -1277,7 +1296,7 @@
       <x:c r="I3" s="102"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="93"/>
+      <x:c r="A4" s="150"/>
       <x:c r="B4" s="90"/>
       <x:c r="C4" s="90"/>
       <x:c r="D4" s="90"/>
@@ -1288,7 +1307,7 @@
       <x:c r="I4" s="102"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="93"/>
+      <x:c r="A5" s="150"/>
       <x:c r="B5" s="90"/>
       <x:c r="C5" s="90"/>
       <x:c r="D5" s="90"/>
@@ -1299,7 +1318,7 @@
       <x:c r="I5" s="102"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="93"/>
+      <x:c r="A6" s="150"/>
       <x:c r="B6" s="90"/>
       <x:c r="C6" s="90"/>
       <x:c r="D6" s="90"/>
@@ -1310,7 +1329,7 @@
       <x:c r="I6" s="102"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="93"/>
+      <x:c r="A7" s="150"/>
       <x:c r="B7" s="90"/>
       <x:c r="C7" s="90"/>
       <x:c r="D7" s="90"/>
@@ -1321,7 +1340,7 @@
       <x:c r="I7" s="102"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="93"/>
+      <x:c r="A8" s="150"/>
       <x:c r="B8" s="90"/>
       <x:c r="C8" s="90"/>
       <x:c r="D8" s="90"/>
@@ -1332,7 +1351,7 @@
       <x:c r="I8" s="102"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="93"/>
+      <x:c r="A9" s="150"/>
       <x:c r="B9" s="90"/>
       <x:c r="C9" s="90"/>
       <x:c r="D9" s="90"/>
@@ -1343,7 +1362,7 @@
       <x:c r="I9" s="102"/>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="93"/>
+      <x:c r="A10" s="150"/>
       <x:c r="B10" s="90"/>
       <x:c r="C10" s="90"/>
       <x:c r="D10" s="90"/>
@@ -1354,7 +1373,7 @@
       <x:c r="I10" s="102"/>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="93"/>
+      <x:c r="A11" s="150"/>
       <x:c r="B11" s="90"/>
       <x:c r="C11" s="90"/>
       <x:c r="D11" s="90"/>
@@ -1365,7 +1384,7 @@
       <x:c r="I11" s="102"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="93"/>
+      <x:c r="A12" s="150"/>
       <x:c r="B12" s="90"/>
       <x:c r="C12" s="90"/>
       <x:c r="D12" s="90"/>
@@ -1376,7 +1395,7 @@
       <x:c r="I12" s="102"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="93"/>
+      <x:c r="A13" s="150"/>
       <x:c r="B13" s="90"/>
       <x:c r="C13" s="90"/>
       <x:c r="D13" s="90"/>
@@ -1387,7 +1406,7 @@
       <x:c r="I13" s="102"/>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="93"/>
+      <x:c r="A14" s="150"/>
       <x:c r="B14" s="90"/>
       <x:c r="C14" s="90"/>
       <x:c r="D14" s="90"/>
@@ -1398,7 +1417,7 @@
       <x:c r="I14" s="102"/>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="93"/>
+      <x:c r="A15" s="150"/>
       <x:c r="B15" s="90"/>
       <x:c r="C15" s="90"/>
       <x:c r="D15" s="90"/>
@@ -1409,7 +1428,7 @@
       <x:c r="I15" s="102"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="93"/>
+      <x:c r="A16" s="150"/>
       <x:c r="B16" s="90"/>
       <x:c r="C16" s="90"/>
       <x:c r="D16" s="90"/>
@@ -1420,7 +1439,7 @@
       <x:c r="I16" s="102"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="93"/>
+      <x:c r="A17" s="150"/>
       <x:c r="B17" s="90"/>
       <x:c r="C17" s="90"/>
       <x:c r="D17" s="90"/>
@@ -1431,7 +1450,7 @@
       <x:c r="I17" s="102"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="93"/>
+      <x:c r="A18" s="150"/>
       <x:c r="B18" s="90"/>
       <x:c r="C18" s="90"/>
       <x:c r="D18" s="90"/>
@@ -1442,7 +1461,7 @@
       <x:c r="I18" s="102"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="93"/>
+      <x:c r="A19" s="150"/>
       <x:c r="B19" s="90"/>
       <x:c r="C19" s="90"/>
       <x:c r="D19" s="90"/>
@@ -1453,7 +1472,7 @@
       <x:c r="I19" s="102"/>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="93"/>
+      <x:c r="A20" s="150"/>
       <x:c r="B20" s="90"/>
       <x:c r="C20" s="90"/>
       <x:c r="D20" s="90"/>
@@ -1464,7 +1483,7 @@
       <x:c r="I20" s="102"/>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="93"/>
+      <x:c r="A21" s="150"/>
       <x:c r="B21" s="90"/>
       <x:c r="C21" s="90"/>
       <x:c r="D21" s="90"/>
@@ -1475,7 +1494,7 @@
       <x:c r="I21" s="102"/>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="93"/>
+      <x:c r="A22" s="150"/>
       <x:c r="B22" s="90"/>
       <x:c r="C22" s="90"/>
       <x:c r="D22" s="90"/>
@@ -1486,7 +1505,7 @@
       <x:c r="I22" s="102"/>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="93"/>
+      <x:c r="A23" s="150"/>
       <x:c r="B23" s="90"/>
       <x:c r="C23" s="90"/>
       <x:c r="D23" s="90"/>
@@ -1497,7 +1516,7 @@
       <x:c r="I23" s="102"/>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="93"/>
+      <x:c r="A24" s="150"/>
       <x:c r="B24" s="90"/>
       <x:c r="C24" s="90"/>
       <x:c r="D24" s="90"/>
@@ -1508,7 +1527,7 @@
       <x:c r="I24" s="102"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="93"/>
+      <x:c r="A25" s="150"/>
       <x:c r="B25" s="90"/>
       <x:c r="C25" s="90"/>
       <x:c r="D25" s="90"/>
@@ -1519,7 +1538,7 @@
       <x:c r="I25" s="102"/>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="93"/>
+      <x:c r="A26" s="150"/>
       <x:c r="B26" s="90"/>
       <x:c r="C26" s="90"/>
       <x:c r="D26" s="90"/>
@@ -1530,7 +1549,7 @@
       <x:c r="I26" s="102"/>
     </x:row>
     <x:row r="27">
-      <x:c r="A27" s="93"/>
+      <x:c r="A27" s="150"/>
       <x:c r="B27" s="90"/>
       <x:c r="C27" s="90"/>
       <x:c r="D27" s="90"/>
@@ -1541,7 +1560,7 @@
       <x:c r="I27" s="102"/>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="93"/>
+      <x:c r="A28" s="150"/>
       <x:c r="B28" s="90"/>
       <x:c r="C28" s="90"/>
       <x:c r="D28" s="90"/>
@@ -1552,7 +1571,7 @@
       <x:c r="I28" s="102"/>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="93"/>
+      <x:c r="A29" s="150"/>
       <x:c r="B29" s="90"/>
       <x:c r="C29" s="90"/>
       <x:c r="D29" s="90"/>
@@ -1563,7 +1582,7 @@
       <x:c r="I29" s="102"/>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="93"/>
+      <x:c r="A30" s="150"/>
       <x:c r="B30" s="90"/>
       <x:c r="C30" s="90"/>
       <x:c r="D30" s="90"/>
@@ -1574,7 +1593,7 @@
       <x:c r="I30" s="102"/>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="93"/>
+      <x:c r="A31" s="150"/>
       <x:c r="B31" s="90"/>
       <x:c r="C31" s="90"/>
       <x:c r="D31" s="90"/>
@@ -1585,7 +1604,7 @@
       <x:c r="I31" s="102"/>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="93"/>
+      <x:c r="A32" s="150"/>
       <x:c r="B32" s="90"/>
       <x:c r="C32" s="90"/>
       <x:c r="D32" s="90"/>
@@ -1596,7 +1615,7 @@
       <x:c r="I32" s="102"/>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" s="93"/>
+      <x:c r="A33" s="150"/>
       <x:c r="B33" s="90"/>
       <x:c r="C33" s="90"/>
       <x:c r="D33" s="90"/>
@@ -1607,7 +1626,7 @@
       <x:c r="I33" s="102"/>
     </x:row>
     <x:row r="34">
-      <x:c r="A34" s="93"/>
+      <x:c r="A34" s="150"/>
       <x:c r="B34" s="90"/>
       <x:c r="C34" s="90"/>
       <x:c r="D34" s="90"/>
@@ -1618,7 +1637,7 @@
       <x:c r="I34" s="102"/>
     </x:row>
     <x:row r="35">
-      <x:c r="A35" s="93"/>
+      <x:c r="A35" s="150"/>
       <x:c r="B35" s="90"/>
       <x:c r="C35" s="90"/>
       <x:c r="D35" s="90"/>
@@ -1629,7 +1648,7 @@
       <x:c r="I35" s="102"/>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" s="93"/>
+      <x:c r="A36" s="150"/>
       <x:c r="B36" s="90"/>
       <x:c r="C36" s="90"/>
       <x:c r="D36" s="90"/>
@@ -1640,7 +1659,7 @@
       <x:c r="I36" s="102"/>
     </x:row>
     <x:row r="37">
-      <x:c r="A37" s="93"/>
+      <x:c r="A37" s="150"/>
       <x:c r="B37" s="90"/>
       <x:c r="C37" s="90"/>
       <x:c r="D37" s="90"/>
@@ -1651,7 +1670,7 @@
       <x:c r="I37" s="102"/>
     </x:row>
     <x:row r="38">
-      <x:c r="A38" s="93"/>
+      <x:c r="A38" s="150"/>
       <x:c r="B38" s="90"/>
       <x:c r="C38" s="90"/>
       <x:c r="D38" s="90"/>
@@ -1662,7 +1681,7 @@
       <x:c r="I38" s="102"/>
     </x:row>
     <x:row r="39">
-      <x:c r="A39" s="93"/>
+      <x:c r="A39" s="150"/>
       <x:c r="B39" s="90"/>
       <x:c r="C39" s="90"/>
       <x:c r="D39" s="90"/>
@@ -1673,7 +1692,7 @@
       <x:c r="I39" s="102"/>
     </x:row>
     <x:row r="40">
-      <x:c r="A40" s="93"/>
+      <x:c r="A40" s="150"/>
       <x:c r="B40" s="90"/>
       <x:c r="C40" s="90"/>
       <x:c r="D40" s="90"/>
@@ -1684,7 +1703,7 @@
       <x:c r="I40" s="102"/>
     </x:row>
     <x:row r="41">
-      <x:c r="A41" s="93"/>
+      <x:c r="A41" s="150"/>
       <x:c r="B41" s="90"/>
       <x:c r="C41" s="90"/>
       <x:c r="D41" s="90"/>
@@ -1695,7 +1714,7 @@
       <x:c r="I41" s="102"/>
     </x:row>
     <x:row r="42">
-      <x:c r="A42" s="93"/>
+      <x:c r="A42" s="150"/>
       <x:c r="B42" s="90"/>
       <x:c r="C42" s="90"/>
       <x:c r="D42" s="90"/>
@@ -1706,7 +1725,7 @@
       <x:c r="I42" s="102"/>
     </x:row>
     <x:row r="43">
-      <x:c r="A43" s="93"/>
+      <x:c r="A43" s="150"/>
       <x:c r="B43" s="90"/>
       <x:c r="C43" s="90"/>
       <x:c r="D43" s="90"/>
@@ -1717,7 +1736,7 @@
       <x:c r="I43" s="102"/>
     </x:row>
     <x:row r="44">
-      <x:c r="A44" s="93"/>
+      <x:c r="A44" s="150"/>
       <x:c r="B44" s="90"/>
       <x:c r="C44" s="90"/>
       <x:c r="D44" s="90"/>
@@ -1728,7 +1747,7 @@
       <x:c r="I44" s="102"/>
     </x:row>
     <x:row r="45">
-      <x:c r="A45" s="93"/>
+      <x:c r="A45" s="150"/>
       <x:c r="B45" s="90"/>
       <x:c r="C45" s="90"/>
       <x:c r="D45" s="90"/>
@@ -1739,7 +1758,7 @@
       <x:c r="I45" s="102"/>
     </x:row>
     <x:row r="46">
-      <x:c r="A46" s="93"/>
+      <x:c r="A46" s="150"/>
       <x:c r="B46" s="90"/>
       <x:c r="C46" s="90"/>
       <x:c r="D46" s="90"/>
@@ -1750,7 +1769,7 @@
       <x:c r="I46" s="102"/>
     </x:row>
     <x:row r="47">
-      <x:c r="A47" s="93"/>
+      <x:c r="A47" s="150"/>
       <x:c r="B47" s="90"/>
       <x:c r="C47" s="90"/>
       <x:c r="D47" s="90"/>
@@ -1761,7 +1780,7 @@
       <x:c r="I47" s="102"/>
     </x:row>
     <x:row r="48">
-      <x:c r="A48" s="93"/>
+      <x:c r="A48" s="150"/>
       <x:c r="B48" s="90"/>
       <x:c r="C48" s="90"/>
       <x:c r="D48" s="90"/>
@@ -1772,7 +1791,7 @@
       <x:c r="I48" s="102"/>
     </x:row>
     <x:row r="49">
-      <x:c r="A49" s="93"/>
+      <x:c r="A49" s="150"/>
       <x:c r="B49" s="90"/>
       <x:c r="C49" s="90"/>
       <x:c r="D49" s="90"/>
@@ -1783,7 +1802,7 @@
       <x:c r="I49" s="102"/>
     </x:row>
     <x:row r="50">
-      <x:c r="A50" s="93"/>
+      <x:c r="A50" s="150"/>
       <x:c r="B50" s="90"/>
       <x:c r="C50" s="90"/>
       <x:c r="D50" s="90"/>
@@ -1794,7 +1813,7 @@
       <x:c r="I50" s="102"/>
     </x:row>
     <x:row r="51">
-      <x:c r="A51" s="93"/>
+      <x:c r="A51" s="150"/>
       <x:c r="B51" s="90"/>
       <x:c r="C51" s="90"/>
       <x:c r="D51" s="90"/>
@@ -1805,7 +1824,7 @@
       <x:c r="I51" s="102"/>
     </x:row>
     <x:row r="52">
-      <x:c r="A52" s="93"/>
+      <x:c r="A52" s="150"/>
       <x:c r="B52" s="90"/>
       <x:c r="C52" s="90"/>
       <x:c r="D52" s="90"/>
@@ -1816,7 +1835,7 @@
       <x:c r="I52" s="102"/>
     </x:row>
     <x:row r="53">
-      <x:c r="A53" s="93"/>
+      <x:c r="A53" s="150"/>
       <x:c r="B53" s="90"/>
       <x:c r="C53" s="90"/>
       <x:c r="D53" s="90"/>
@@ -1827,7 +1846,7 @@
       <x:c r="I53" s="102"/>
     </x:row>
     <x:row r="54">
-      <x:c r="A54" s="93"/>
+      <x:c r="A54" s="150"/>
       <x:c r="B54" s="90"/>
       <x:c r="C54" s="90"/>
       <x:c r="D54" s="90"/>
@@ -1838,7 +1857,7 @@
       <x:c r="I54" s="102"/>
     </x:row>
     <x:row r="55">
-      <x:c r="A55" s="93"/>
+      <x:c r="A55" s="150"/>
       <x:c r="B55" s="90"/>
       <x:c r="C55" s="90"/>
       <x:c r="D55" s="90"/>
@@ -1849,7 +1868,7 @@
       <x:c r="I55" s="102"/>
     </x:row>
     <x:row r="56">
-      <x:c r="A56" s="93"/>
+      <x:c r="A56" s="150"/>
       <x:c r="B56" s="90"/>
       <x:c r="C56" s="90"/>
       <x:c r="D56" s="90"/>
@@ -1860,7 +1879,7 @@
       <x:c r="I56" s="102"/>
     </x:row>
     <x:row r="57">
-      <x:c r="A57" s="93"/>
+      <x:c r="A57" s="150"/>
       <x:c r="B57" s="90"/>
       <x:c r="C57" s="90"/>
       <x:c r="D57" s="90"/>
@@ -1871,7 +1890,7 @@
       <x:c r="I57" s="102"/>
     </x:row>
     <x:row r="58">
-      <x:c r="A58" s="93"/>
+      <x:c r="A58" s="150"/>
       <x:c r="B58" s="90"/>
       <x:c r="C58" s="90"/>
       <x:c r="D58" s="90"/>
@@ -1882,7 +1901,7 @@
       <x:c r="I58" s="102"/>
     </x:row>
     <x:row r="59">
-      <x:c r="A59" s="93"/>
+      <x:c r="A59" s="150"/>
       <x:c r="B59" s="90"/>
       <x:c r="C59" s="90"/>
       <x:c r="D59" s="90"/>
@@ -1893,7 +1912,7 @@
       <x:c r="I59" s="102"/>
     </x:row>
     <x:row r="60">
-      <x:c r="A60" s="93"/>
+      <x:c r="A60" s="150"/>
       <x:c r="B60" s="90"/>
       <x:c r="C60" s="90"/>
       <x:c r="D60" s="90"/>
@@ -1904,7 +1923,7 @@
       <x:c r="I60" s="102"/>
     </x:row>
     <x:row r="61">
-      <x:c r="A61" s="93"/>
+      <x:c r="A61" s="150"/>
       <x:c r="B61" s="90"/>
       <x:c r="C61" s="90"/>
       <x:c r="D61" s="90"/>
@@ -1915,7 +1934,7 @@
       <x:c r="I61" s="102"/>
     </x:row>
     <x:row r="62">
-      <x:c r="A62" s="93"/>
+      <x:c r="A62" s="150"/>
       <x:c r="B62" s="90"/>
       <x:c r="C62" s="90"/>
       <x:c r="D62" s="90"/>
@@ -1926,7 +1945,7 @@
       <x:c r="I62" s="102"/>
     </x:row>
     <x:row r="63">
-      <x:c r="A63" s="93"/>
+      <x:c r="A63" s="150"/>
       <x:c r="B63" s="90"/>
       <x:c r="C63" s="90"/>
       <x:c r="D63" s="90"/>
@@ -1937,7 +1956,7 @@
       <x:c r="I63" s="102"/>
     </x:row>
     <x:row r="64">
-      <x:c r="A64" s="93"/>
+      <x:c r="A64" s="150"/>
       <x:c r="B64" s="90"/>
       <x:c r="C64" s="90"/>
       <x:c r="D64" s="90"/>
@@ -1948,7 +1967,7 @@
       <x:c r="I64" s="102"/>
     </x:row>
     <x:row r="65">
-      <x:c r="A65" s="93"/>
+      <x:c r="A65" s="150"/>
       <x:c r="B65" s="90"/>
       <x:c r="C65" s="90"/>
       <x:c r="D65" s="90"/>
@@ -1959,7 +1978,7 @@
       <x:c r="I65" s="102"/>
     </x:row>
     <x:row r="66">
-      <x:c r="A66" s="93"/>
+      <x:c r="A66" s="150"/>
       <x:c r="B66" s="90"/>
       <x:c r="C66" s="90"/>
       <x:c r="D66" s="90"/>
@@ -1970,7 +1989,7 @@
       <x:c r="I66" s="102"/>
     </x:row>
     <x:row r="67">
-      <x:c r="A67" s="93"/>
+      <x:c r="A67" s="150"/>
       <x:c r="B67" s="90"/>
       <x:c r="C67" s="90"/>
       <x:c r="D67" s="90"/>
@@ -1981,7 +2000,7 @@
       <x:c r="I67" s="102"/>
     </x:row>
     <x:row r="68">
-      <x:c r="A68" s="93"/>
+      <x:c r="A68" s="150"/>
       <x:c r="B68" s="90"/>
       <x:c r="C68" s="90"/>
       <x:c r="D68" s="90"/>
@@ -1992,7 +2011,7 @@
       <x:c r="I68" s="102"/>
     </x:row>
     <x:row r="69">
-      <x:c r="A69" s="93"/>
+      <x:c r="A69" s="150"/>
       <x:c r="B69" s="90"/>
       <x:c r="C69" s="90"/>
       <x:c r="D69" s="90"/>
@@ -2003,7 +2022,7 @@
       <x:c r="I69" s="102"/>
     </x:row>
     <x:row r="70">
-      <x:c r="A70" s="93"/>
+      <x:c r="A70" s="150"/>
       <x:c r="B70" s="90"/>
       <x:c r="C70" s="90"/>
       <x:c r="D70" s="90"/>
@@ -2014,7 +2033,7 @@
       <x:c r="I70" s="102"/>
     </x:row>
     <x:row r="71">
-      <x:c r="A71" s="93"/>
+      <x:c r="A71" s="150"/>
       <x:c r="B71" s="90"/>
       <x:c r="C71" s="90"/>
       <x:c r="D71" s="90"/>
@@ -2025,7 +2044,7 @@
       <x:c r="I71" s="102"/>
     </x:row>
     <x:row r="72">
-      <x:c r="A72" s="93"/>
+      <x:c r="A72" s="150"/>
       <x:c r="B72" s="90"/>
       <x:c r="C72" s="90"/>
       <x:c r="D72" s="90"/>
@@ -2036,7 +2055,7 @@
       <x:c r="I72" s="102"/>
     </x:row>
     <x:row r="73">
-      <x:c r="A73" s="93"/>
+      <x:c r="A73" s="150"/>
       <x:c r="B73" s="90"/>
       <x:c r="C73" s="90"/>
       <x:c r="D73" s="90"/>
@@ -2047,7 +2066,7 @@
       <x:c r="I73" s="102"/>
     </x:row>
     <x:row r="74">
-      <x:c r="A74" s="93"/>
+      <x:c r="A74" s="150"/>
       <x:c r="B74" s="90"/>
       <x:c r="C74" s="90"/>
       <x:c r="D74" s="90"/>
@@ -2058,7 +2077,7 @@
       <x:c r="I74" s="102"/>
     </x:row>
     <x:row r="75">
-      <x:c r="A75" s="93"/>
+      <x:c r="A75" s="150"/>
       <x:c r="B75" s="90"/>
       <x:c r="C75" s="90"/>
       <x:c r="D75" s="90"/>
@@ -2069,7 +2088,7 @@
       <x:c r="I75" s="102"/>
     </x:row>
     <x:row r="76">
-      <x:c r="A76" s="93"/>
+      <x:c r="A76" s="150"/>
       <x:c r="B76" s="90"/>
       <x:c r="C76" s="90"/>
       <x:c r="D76" s="90"/>
@@ -2080,7 +2099,7 @@
       <x:c r="I76" s="102"/>
     </x:row>
     <x:row r="77">
-      <x:c r="A77" s="93"/>
+      <x:c r="A77" s="150"/>
       <x:c r="B77" s="90"/>
       <x:c r="C77" s="90"/>
       <x:c r="D77" s="90"/>
@@ -2091,7 +2110,7 @@
       <x:c r="I77" s="102"/>
     </x:row>
     <x:row r="78">
-      <x:c r="A78" s="93"/>
+      <x:c r="A78" s="150"/>
       <x:c r="B78" s="90"/>
       <x:c r="C78" s="90"/>
       <x:c r="D78" s="90"/>
@@ -2102,7 +2121,7 @@
       <x:c r="I78" s="102"/>
     </x:row>
     <x:row r="79">
-      <x:c r="A79" s="93"/>
+      <x:c r="A79" s="150"/>
       <x:c r="B79" s="90"/>
       <x:c r="C79" s="90"/>
       <x:c r="D79" s="90"/>
@@ -2113,7 +2132,7 @@
       <x:c r="I79" s="102"/>
     </x:row>
     <x:row r="80">
-      <x:c r="A80" s="93"/>
+      <x:c r="A80" s="150"/>
       <x:c r="B80" s="90"/>
       <x:c r="C80" s="90"/>
       <x:c r="D80" s="90"/>
@@ -2124,7 +2143,7 @@
       <x:c r="I80" s="102"/>
     </x:row>
     <x:row r="81">
-      <x:c r="A81" s="93"/>
+      <x:c r="A81" s="150"/>
       <x:c r="B81" s="90"/>
       <x:c r="C81" s="90"/>
       <x:c r="D81" s="90"/>
@@ -2135,7 +2154,7 @@
       <x:c r="I81" s="102"/>
     </x:row>
     <x:row r="82">
-      <x:c r="A82" s="93"/>
+      <x:c r="A82" s="150"/>
       <x:c r="B82" s="90"/>
       <x:c r="C82" s="90"/>
       <x:c r="D82" s="90"/>
@@ -2146,7 +2165,7 @@
       <x:c r="I82" s="102"/>
     </x:row>
     <x:row r="83">
-      <x:c r="A83" s="93"/>
+      <x:c r="A83" s="150"/>
       <x:c r="B83" s="90"/>
       <x:c r="C83" s="90"/>
       <x:c r="D83" s="90"/>
@@ -2157,7 +2176,7 @@
       <x:c r="I83" s="102"/>
     </x:row>
     <x:row r="84">
-      <x:c r="A84" s="93"/>
+      <x:c r="A84" s="150"/>
       <x:c r="B84" s="90"/>
       <x:c r="C84" s="90"/>
       <x:c r="D84" s="90"/>
@@ -2168,7 +2187,7 @@
       <x:c r="I84" s="102"/>
     </x:row>
     <x:row r="85">
-      <x:c r="A85" s="93"/>
+      <x:c r="A85" s="150"/>
       <x:c r="B85" s="90"/>
       <x:c r="C85" s="90"/>
       <x:c r="D85" s="90"/>
@@ -2179,7 +2198,7 @@
       <x:c r="I85" s="102"/>
     </x:row>
     <x:row r="86">
-      <x:c r="A86" s="93"/>
+      <x:c r="A86" s="150"/>
       <x:c r="B86" s="90"/>
       <x:c r="C86" s="90"/>
       <x:c r="D86" s="90"/>
@@ -2190,7 +2209,7 @@
       <x:c r="I86" s="102"/>
     </x:row>
     <x:row r="87">
-      <x:c r="A87" s="93"/>
+      <x:c r="A87" s="150"/>
       <x:c r="B87" s="90"/>
       <x:c r="C87" s="90"/>
       <x:c r="D87" s="90"/>
@@ -2201,7 +2220,7 @@
       <x:c r="I87" s="102"/>
     </x:row>
     <x:row r="88">
-      <x:c r="A88" s="93"/>
+      <x:c r="A88" s="150"/>
       <x:c r="B88" s="90"/>
       <x:c r="C88" s="90"/>
       <x:c r="D88" s="90"/>
@@ -2212,7 +2231,7 @@
       <x:c r="I88" s="102"/>
     </x:row>
     <x:row r="89">
-      <x:c r="A89" s="93"/>
+      <x:c r="A89" s="150"/>
       <x:c r="B89" s="90"/>
       <x:c r="C89" s="90"/>
       <x:c r="D89" s="90"/>
@@ -2223,7 +2242,7 @@
       <x:c r="I89" s="102"/>
     </x:row>
     <x:row r="90">
-      <x:c r="A90" s="93"/>
+      <x:c r="A90" s="150"/>
       <x:c r="B90" s="90"/>
       <x:c r="C90" s="90"/>
       <x:c r="D90" s="90"/>
@@ -2234,7 +2253,7 @@
       <x:c r="I90" s="102"/>
     </x:row>
     <x:row r="91">
-      <x:c r="A91" s="93"/>
+      <x:c r="A91" s="150"/>
       <x:c r="B91" s="90"/>
       <x:c r="C91" s="90"/>
       <x:c r="D91" s="90"/>
@@ -2245,7 +2264,7 @@
       <x:c r="I91" s="102"/>
     </x:row>
     <x:row r="92">
-      <x:c r="A92" s="93"/>
+      <x:c r="A92" s="150"/>
       <x:c r="B92" s="90"/>
       <x:c r="C92" s="90"/>
       <x:c r="D92" s="90"/>
@@ -2256,7 +2275,7 @@
       <x:c r="I92" s="102"/>
     </x:row>
     <x:row r="93">
-      <x:c r="A93" s="93"/>
+      <x:c r="A93" s="150"/>
       <x:c r="B93" s="90"/>
       <x:c r="C93" s="90"/>
       <x:c r="D93" s="90"/>
@@ -2267,7 +2286,7 @@
       <x:c r="I93" s="102"/>
     </x:row>
     <x:row r="94">
-      <x:c r="A94" s="93"/>
+      <x:c r="A94" s="150"/>
       <x:c r="B94" s="90"/>
       <x:c r="C94" s="90"/>
       <x:c r="D94" s="90"/>
@@ -2278,7 +2297,7 @@
       <x:c r="I94" s="102"/>
     </x:row>
     <x:row r="95">
-      <x:c r="A95" s="93"/>
+      <x:c r="A95" s="150"/>
       <x:c r="B95" s="90"/>
       <x:c r="C95" s="90"/>
       <x:c r="D95" s="90"/>
@@ -2289,7 +2308,7 @@
       <x:c r="I95" s="102"/>
     </x:row>
     <x:row r="96">
-      <x:c r="A96" s="93"/>
+      <x:c r="A96" s="150"/>
       <x:c r="B96" s="90"/>
       <x:c r="C96" s="90"/>
       <x:c r="D96" s="90"/>
@@ -2300,7 +2319,7 @@
       <x:c r="I96" s="102"/>
     </x:row>
     <x:row r="97">
-      <x:c r="A97" s="93"/>
+      <x:c r="A97" s="150"/>
       <x:c r="B97" s="90"/>
       <x:c r="C97" s="90"/>
       <x:c r="D97" s="90"/>
@@ -2311,7 +2330,7 @@
       <x:c r="I97" s="102"/>
     </x:row>
     <x:row r="98">
-      <x:c r="A98" s="93"/>
+      <x:c r="A98" s="150"/>
       <x:c r="B98" s="90"/>
       <x:c r="C98" s="90"/>
       <x:c r="D98" s="90"/>
@@ -2322,7 +2341,7 @@
       <x:c r="I98" s="102"/>
     </x:row>
     <x:row r="99">
-      <x:c r="A99" s="93"/>
+      <x:c r="A99" s="150"/>
       <x:c r="B99" s="90"/>
       <x:c r="C99" s="90"/>
       <x:c r="D99" s="90"/>
@@ -2333,7 +2352,7 @@
       <x:c r="I99" s="102"/>
     </x:row>
     <x:row r="100">
-      <x:c r="A100" s="93"/>
+      <x:c r="A100" s="150"/>
       <x:c r="B100" s="90"/>
       <x:c r="C100" s="90"/>
       <x:c r="D100" s="90"/>
@@ -2344,7 +2363,7 @@
       <x:c r="I100" s="102"/>
     </x:row>
     <x:row r="101">
-      <x:c r="A101" s="93"/>
+      <x:c r="A101" s="150"/>
       <x:c r="B101" s="90"/>
       <x:c r="C101" s="90"/>
       <x:c r="D101" s="90"/>
@@ -2355,7 +2374,7 @@
       <x:c r="I101" s="102"/>
     </x:row>
     <x:row r="102">
-      <x:c r="A102" s="93"/>
+      <x:c r="A102" s="150"/>
       <x:c r="B102" s="90"/>
       <x:c r="C102" s="90"/>
       <x:c r="D102" s="90"/>
@@ -2366,7 +2385,7 @@
       <x:c r="I102" s="102"/>
     </x:row>
     <x:row r="103">
-      <x:c r="A103" s="93"/>
+      <x:c r="A103" s="150"/>
       <x:c r="B103" s="90"/>
       <x:c r="C103" s="90"/>
       <x:c r="D103" s="90"/>
@@ -2377,7 +2396,7 @@
       <x:c r="I103" s="102"/>
     </x:row>
     <x:row r="104">
-      <x:c r="A104" s="93"/>
+      <x:c r="A104" s="150"/>
       <x:c r="B104" s="90"/>
       <x:c r="C104" s="90"/>
       <x:c r="D104" s="90"/>
@@ -2388,7 +2407,7 @@
       <x:c r="I104" s="102"/>
     </x:row>
     <x:row r="105">
-      <x:c r="A105" s="93"/>
+      <x:c r="A105" s="150"/>
       <x:c r="B105" s="90"/>
       <x:c r="C105" s="90"/>
       <x:c r="D105" s="90"/>
@@ -2399,7 +2418,7 @@
       <x:c r="I105" s="102"/>
     </x:row>
     <x:row r="106">
-      <x:c r="A106" s="93"/>
+      <x:c r="A106" s="150"/>
       <x:c r="B106" s="90"/>
       <x:c r="C106" s="90"/>
       <x:c r="D106" s="90"/>
@@ -2410,7 +2429,7 @@
       <x:c r="I106" s="102"/>
     </x:row>
     <x:row r="107">
-      <x:c r="A107" s="93"/>
+      <x:c r="A107" s="150"/>
       <x:c r="B107" s="90"/>
       <x:c r="C107" s="90"/>
       <x:c r="D107" s="90"/>
@@ -2421,7 +2440,7 @@
       <x:c r="I107" s="102"/>
     </x:row>
     <x:row r="108">
-      <x:c r="A108" s="93"/>
+      <x:c r="A108" s="150"/>
       <x:c r="B108" s="90"/>
       <x:c r="C108" s="90"/>
       <x:c r="D108" s="90"/>
@@ -2432,7 +2451,7 @@
       <x:c r="I108" s="102"/>
     </x:row>
     <x:row r="109">
-      <x:c r="A109" s="93"/>
+      <x:c r="A109" s="150"/>
       <x:c r="B109" s="90"/>
       <x:c r="C109" s="90"/>
       <x:c r="D109" s="90"/>
@@ -2443,7 +2462,7 @@
       <x:c r="I109" s="102"/>
     </x:row>
     <x:row r="110">
-      <x:c r="A110" s="93"/>
+      <x:c r="A110" s="150"/>
       <x:c r="B110" s="90"/>
       <x:c r="C110" s="90"/>
       <x:c r="D110" s="90"/>
@@ -2454,7 +2473,7 @@
       <x:c r="I110" s="102"/>
     </x:row>
     <x:row r="111">
-      <x:c r="A111" s="93"/>
+      <x:c r="A111" s="150"/>
       <x:c r="B111" s="90"/>
       <x:c r="C111" s="90"/>
       <x:c r="D111" s="90"/>
@@ -2465,7 +2484,7 @@
       <x:c r="I111" s="102"/>
     </x:row>
     <x:row r="112">
-      <x:c r="A112" s="93"/>
+      <x:c r="A112" s="150"/>
       <x:c r="B112" s="90"/>
       <x:c r="C112" s="90"/>
       <x:c r="D112" s="90"/>
@@ -2476,7 +2495,7 @@
       <x:c r="I112" s="102"/>
     </x:row>
     <x:row r="113">
-      <x:c r="A113" s="93"/>
+      <x:c r="A113" s="150"/>
       <x:c r="B113" s="90"/>
       <x:c r="C113" s="90"/>
       <x:c r="D113" s="90"/>
@@ -2487,7 +2506,7 @@
       <x:c r="I113" s="102"/>
     </x:row>
     <x:row r="114">
-      <x:c r="A114" s="93"/>
+      <x:c r="A114" s="150"/>
       <x:c r="B114" s="90"/>
       <x:c r="C114" s="90"/>
       <x:c r="D114" s="90"/>
@@ -2498,7 +2517,7 @@
       <x:c r="I114" s="102"/>
     </x:row>
     <x:row r="115">
-      <x:c r="A115" s="93"/>
+      <x:c r="A115" s="150"/>
       <x:c r="B115" s="90"/>
       <x:c r="C115" s="90"/>
       <x:c r="D115" s="90"/>
@@ -2509,7 +2528,7 @@
       <x:c r="I115" s="102"/>
     </x:row>
     <x:row r="116">
-      <x:c r="A116" s="93"/>
+      <x:c r="A116" s="150"/>
       <x:c r="B116" s="90"/>
       <x:c r="C116" s="90"/>
       <x:c r="D116" s="90"/>
@@ -2520,7 +2539,7 @@
       <x:c r="I116" s="102"/>
     </x:row>
     <x:row r="117">
-      <x:c r="A117" s="93"/>
+      <x:c r="A117" s="150"/>
       <x:c r="B117" s="90"/>
       <x:c r="C117" s="90"/>
       <x:c r="D117" s="90"/>
@@ -2531,7 +2550,7 @@
       <x:c r="I117" s="102"/>
     </x:row>
     <x:row r="118">
-      <x:c r="A118" s="93"/>
+      <x:c r="A118" s="150"/>
       <x:c r="B118" s="90"/>
       <x:c r="C118" s="90"/>
       <x:c r="D118" s="90"/>
@@ -2542,7 +2561,7 @@
       <x:c r="I118" s="102"/>
     </x:row>
     <x:row r="119">
-      <x:c r="A119" s="93"/>
+      <x:c r="A119" s="150"/>
       <x:c r="B119" s="90"/>
       <x:c r="C119" s="90"/>
       <x:c r="D119" s="90"/>
@@ -2553,7 +2572,7 @@
       <x:c r="I119" s="102"/>
     </x:row>
     <x:row r="120">
-      <x:c r="A120" s="93"/>
+      <x:c r="A120" s="150"/>
       <x:c r="B120" s="90"/>
       <x:c r="C120" s="90"/>
       <x:c r="D120" s="90"/>
@@ -2564,7 +2583,7 @@
       <x:c r="I120" s="102"/>
     </x:row>
     <x:row r="121">
-      <x:c r="A121" s="93"/>
+      <x:c r="A121" s="150"/>
       <x:c r="B121" s="90"/>
       <x:c r="C121" s="90"/>
       <x:c r="D121" s="90"/>
@@ -2575,7 +2594,7 @@
       <x:c r="I121" s="102"/>
     </x:row>
     <x:row r="122">
-      <x:c r="A122" s="93"/>
+      <x:c r="A122" s="150"/>
       <x:c r="B122" s="90"/>
       <x:c r="C122" s="90"/>
       <x:c r="D122" s="90"/>
@@ -2586,7 +2605,7 @@
       <x:c r="I122" s="102"/>
     </x:row>
     <x:row r="123">
-      <x:c r="A123" s="93"/>
+      <x:c r="A123" s="150"/>
       <x:c r="B123" s="90"/>
       <x:c r="C123" s="90"/>
       <x:c r="D123" s="90"/>
@@ -2597,7 +2616,7 @@
       <x:c r="I123" s="102"/>
     </x:row>
     <x:row r="124">
-      <x:c r="A124" s="93"/>
+      <x:c r="A124" s="150"/>
       <x:c r="B124" s="90"/>
       <x:c r="C124" s="90"/>
       <x:c r="D124" s="90"/>
@@ -2608,7 +2627,7 @@
       <x:c r="I124" s="102"/>
     </x:row>
     <x:row r="125">
-      <x:c r="A125" s="93"/>
+      <x:c r="A125" s="150"/>
       <x:c r="B125" s="90"/>
       <x:c r="C125" s="90"/>
       <x:c r="D125" s="90"/>
@@ -2619,7 +2638,7 @@
       <x:c r="I125" s="102"/>
     </x:row>
     <x:row r="126">
-      <x:c r="A126" s="93"/>
+      <x:c r="A126" s="150"/>
       <x:c r="B126" s="90"/>
       <x:c r="C126" s="90"/>
       <x:c r="D126" s="90"/>
@@ -2630,7 +2649,7 @@
       <x:c r="I126" s="102"/>
     </x:row>
     <x:row r="127">
-      <x:c r="A127" s="93"/>
+      <x:c r="A127" s="150"/>
       <x:c r="B127" s="90"/>
       <x:c r="C127" s="90"/>
       <x:c r="D127" s="90"/>
@@ -2641,7 +2660,7 @@
       <x:c r="I127" s="102"/>
     </x:row>
     <x:row r="128">
-      <x:c r="A128" s="93"/>
+      <x:c r="A128" s="150"/>
       <x:c r="B128" s="90"/>
       <x:c r="C128" s="90"/>
       <x:c r="D128" s="90"/>
@@ -2652,7 +2671,7 @@
       <x:c r="I128" s="102"/>
     </x:row>
     <x:row r="129">
-      <x:c r="A129" s="93"/>
+      <x:c r="A129" s="150"/>
       <x:c r="B129" s="90"/>
       <x:c r="C129" s="90"/>
       <x:c r="D129" s="90"/>
@@ -2663,7 +2682,7 @@
       <x:c r="I129" s="102"/>
     </x:row>
     <x:row r="130">
-      <x:c r="A130" s="93"/>
+      <x:c r="A130" s="150"/>
       <x:c r="B130" s="90"/>
       <x:c r="C130" s="90"/>
       <x:c r="D130" s="90"/>
@@ -2674,7 +2693,7 @@
       <x:c r="I130" s="102"/>
     </x:row>
     <x:row r="131">
-      <x:c r="A131" s="93"/>
+      <x:c r="A131" s="150"/>
       <x:c r="B131" s="90"/>
       <x:c r="C131" s="90"/>
       <x:c r="D131" s="90"/>
@@ -2685,7 +2704,7 @@
       <x:c r="I131" s="102"/>
     </x:row>
     <x:row r="132">
-      <x:c r="A132" s="93"/>
+      <x:c r="A132" s="150"/>
       <x:c r="B132" s="90"/>
       <x:c r="C132" s="90"/>
       <x:c r="D132" s="90"/>
@@ -2696,7 +2715,7 @@
       <x:c r="I132" s="102"/>
     </x:row>
     <x:row r="133">
-      <x:c r="A133" s="93"/>
+      <x:c r="A133" s="150"/>
       <x:c r="B133" s="90"/>
       <x:c r="C133" s="90"/>
       <x:c r="D133" s="90"/>
@@ -2707,7 +2726,7 @@
       <x:c r="I133" s="102"/>
     </x:row>
     <x:row r="134">
-      <x:c r="A134" s="93"/>
+      <x:c r="A134" s="150"/>
       <x:c r="B134" s="90"/>
       <x:c r="C134" s="90"/>
       <x:c r="D134" s="90"/>
@@ -2718,7 +2737,7 @@
       <x:c r="I134" s="102"/>
     </x:row>
     <x:row r="135">
-      <x:c r="A135" s="93"/>
+      <x:c r="A135" s="150"/>
       <x:c r="B135" s="90"/>
       <x:c r="C135" s="90"/>
       <x:c r="D135" s="90"/>
@@ -2729,7 +2748,7 @@
       <x:c r="I135" s="102"/>
     </x:row>
     <x:row r="136">
-      <x:c r="A136" s="93"/>
+      <x:c r="A136" s="150"/>
       <x:c r="B136" s="90"/>
       <x:c r="C136" s="90"/>
       <x:c r="D136" s="90"/>
@@ -2740,7 +2759,7 @@
       <x:c r="I136" s="102"/>
     </x:row>
     <x:row r="137">
-      <x:c r="A137" s="93"/>
+      <x:c r="A137" s="150"/>
       <x:c r="B137" s="90"/>
       <x:c r="C137" s="90"/>
       <x:c r="D137" s="90"/>
@@ -2751,7 +2770,7 @@
       <x:c r="I137" s="102"/>
     </x:row>
     <x:row r="138">
-      <x:c r="A138" s="93"/>
+      <x:c r="A138" s="150"/>
       <x:c r="B138" s="90"/>
       <x:c r="C138" s="90"/>
       <x:c r="D138" s="90"/>
@@ -2762,7 +2781,7 @@
       <x:c r="I138" s="102"/>
     </x:row>
     <x:row r="139">
-      <x:c r="A139" s="93"/>
+      <x:c r="A139" s="150"/>
       <x:c r="B139" s="90"/>
       <x:c r="C139" s="90"/>
       <x:c r="D139" s="90"/>
@@ -2773,7 +2792,7 @@
       <x:c r="I139" s="102"/>
     </x:row>
     <x:row r="140">
-      <x:c r="A140" s="93"/>
+      <x:c r="A140" s="150"/>
       <x:c r="B140" s="90"/>
       <x:c r="C140" s="90"/>
       <x:c r="D140" s="90"/>
@@ -2784,7 +2803,7 @@
       <x:c r="I140" s="102"/>
     </x:row>
     <x:row r="141">
-      <x:c r="A141" s="93"/>
+      <x:c r="A141" s="150"/>
       <x:c r="B141" s="90"/>
       <x:c r="C141" s="90"/>
       <x:c r="D141" s="90"/>
@@ -2795,7 +2814,7 @@
       <x:c r="I141" s="102"/>
     </x:row>
     <x:row r="142">
-      <x:c r="A142" s="93"/>
+      <x:c r="A142" s="150"/>
       <x:c r="B142" s="90"/>
       <x:c r="C142" s="90"/>
       <x:c r="D142" s="90"/>
@@ -2806,7 +2825,7 @@
       <x:c r="I142" s="102"/>
     </x:row>
     <x:row r="143">
-      <x:c r="A143" s="93"/>
+      <x:c r="A143" s="150"/>
       <x:c r="B143" s="90"/>
       <x:c r="C143" s="90"/>
       <x:c r="D143" s="90"/>
@@ -2817,7 +2836,7 @@
       <x:c r="I143" s="102"/>
     </x:row>
     <x:row r="144">
-      <x:c r="A144" s="93"/>
+      <x:c r="A144" s="150"/>
       <x:c r="B144" s="90"/>
       <x:c r="C144" s="90"/>
       <x:c r="D144" s="90"/>
@@ -2828,7 +2847,7 @@
       <x:c r="I144" s="102"/>
     </x:row>
     <x:row r="145">
-      <x:c r="A145" s="93"/>
+      <x:c r="A145" s="150"/>
       <x:c r="B145" s="90"/>
       <x:c r="C145" s="90"/>
       <x:c r="D145" s="90"/>
@@ -2839,7 +2858,7 @@
       <x:c r="I145" s="102"/>
     </x:row>
     <x:row r="146">
-      <x:c r="A146" s="93"/>
+      <x:c r="A146" s="150"/>
       <x:c r="B146" s="90"/>
       <x:c r="C146" s="90"/>
       <x:c r="D146" s="90"/>
@@ -2850,7 +2869,7 @@
       <x:c r="I146" s="102"/>
     </x:row>
     <x:row r="147">
-      <x:c r="A147" s="93"/>
+      <x:c r="A147" s="150"/>
       <x:c r="B147" s="90"/>
       <x:c r="C147" s="90"/>
       <x:c r="D147" s="90"/>
@@ -2861,7 +2880,7 @@
       <x:c r="I147" s="102"/>
     </x:row>
     <x:row r="148">
-      <x:c r="A148" s="93"/>
+      <x:c r="A148" s="150"/>
       <x:c r="B148" s="90"/>
       <x:c r="C148" s="90"/>
       <x:c r="D148" s="90"/>
@@ -2872,7 +2891,7 @@
       <x:c r="I148" s="102"/>
     </x:row>
     <x:row r="149">
-      <x:c r="A149" s="93"/>
+      <x:c r="A149" s="150"/>
       <x:c r="B149" s="90"/>
       <x:c r="C149" s="90"/>
       <x:c r="D149" s="90"/>
@@ -2883,7 +2902,7 @@
       <x:c r="I149" s="102"/>
     </x:row>
     <x:row r="150">
-      <x:c r="A150" s="93"/>
+      <x:c r="A150" s="150"/>
       <x:c r="B150" s="90"/>
       <x:c r="C150" s="90"/>
       <x:c r="D150" s="90"/>
@@ -2894,7 +2913,7 @@
       <x:c r="I150" s="102"/>
     </x:row>
     <x:row r="151">
-      <x:c r="A151" s="93"/>
+      <x:c r="A151" s="150"/>
       <x:c r="B151" s="90"/>
       <x:c r="C151" s="90"/>
       <x:c r="D151" s="90"/>
@@ -2905,7 +2924,7 @@
       <x:c r="I151" s="102"/>
     </x:row>
     <x:row r="152">
-      <x:c r="A152" s="93"/>
+      <x:c r="A152" s="150"/>
       <x:c r="B152" s="90"/>
       <x:c r="C152" s="90"/>
       <x:c r="D152" s="90"/>
@@ -2916,7 +2935,7 @@
       <x:c r="I152" s="102"/>
     </x:row>
     <x:row r="153">
-      <x:c r="A153" s="93"/>
+      <x:c r="A153" s="150"/>
       <x:c r="B153" s="90"/>
       <x:c r="C153" s="90"/>
       <x:c r="D153" s="90"/>
@@ -2927,7 +2946,7 @@
       <x:c r="I153" s="102"/>
     </x:row>
     <x:row r="154">
-      <x:c r="A154" s="93"/>
+      <x:c r="A154" s="150"/>
       <x:c r="B154" s="90"/>
       <x:c r="C154" s="90"/>
       <x:c r="D154" s="90"/>
@@ -2938,7 +2957,7 @@
       <x:c r="I154" s="102"/>
     </x:row>
     <x:row r="155">
-      <x:c r="A155" s="93"/>
+      <x:c r="A155" s="150"/>
       <x:c r="B155" s="90"/>
       <x:c r="C155" s="90"/>
       <x:c r="D155" s="90"/>
@@ -2949,7 +2968,7 @@
       <x:c r="I155" s="102"/>
     </x:row>
     <x:row r="156">
-      <x:c r="A156" s="93"/>
+      <x:c r="A156" s="150"/>
       <x:c r="B156" s="90"/>
       <x:c r="C156" s="90"/>
       <x:c r="D156" s="90"/>
@@ -2960,7 +2979,7 @@
       <x:c r="I156" s="102"/>
     </x:row>
     <x:row r="157">
-      <x:c r="A157" s="93"/>
+      <x:c r="A157" s="150"/>
       <x:c r="B157" s="90"/>
       <x:c r="C157" s="90"/>
       <x:c r="D157" s="90"/>
@@ -2971,7 +2990,7 @@
       <x:c r="I157" s="102"/>
     </x:row>
     <x:row r="158">
-      <x:c r="A158" s="93"/>
+      <x:c r="A158" s="150"/>
       <x:c r="B158" s="90"/>
       <x:c r="C158" s="90"/>
       <x:c r="D158" s="90"/>
@@ -2982,7 +3001,7 @@
       <x:c r="I158" s="102"/>
     </x:row>
     <x:row r="159">
-      <x:c r="A159" s="93"/>
+      <x:c r="A159" s="150"/>
       <x:c r="B159" s="90"/>
       <x:c r="C159" s="90"/>
       <x:c r="D159" s="90"/>
@@ -2993,7 +3012,7 @@
       <x:c r="I159" s="102"/>
     </x:row>
     <x:row r="160">
-      <x:c r="A160" s="93"/>
+      <x:c r="A160" s="150"/>
       <x:c r="B160" s="90"/>
       <x:c r="C160" s="90"/>
       <x:c r="D160" s="90"/>
@@ -3004,7 +3023,7 @@
       <x:c r="I160" s="102"/>
     </x:row>
     <x:row r="161">
-      <x:c r="A161" s="93"/>
+      <x:c r="A161" s="150"/>
       <x:c r="B161" s="90"/>
       <x:c r="C161" s="90"/>
       <x:c r="D161" s="90"/>
@@ -3015,7 +3034,7 @@
       <x:c r="I161" s="102"/>
     </x:row>
     <x:row r="162">
-      <x:c r="A162" s="93"/>
+      <x:c r="A162" s="150"/>
       <x:c r="B162" s="90"/>
       <x:c r="C162" s="90"/>
       <x:c r="D162" s="90"/>
@@ -3026,7 +3045,7 @@
       <x:c r="I162" s="102"/>
     </x:row>
     <x:row r="163">
-      <x:c r="A163" s="93"/>
+      <x:c r="A163" s="150"/>
       <x:c r="B163" s="90"/>
       <x:c r="C163" s="90"/>
       <x:c r="D163" s="90"/>
@@ -3037,7 +3056,7 @@
       <x:c r="I163" s="102"/>
     </x:row>
     <x:row r="164">
-      <x:c r="A164" s="93"/>
+      <x:c r="A164" s="150"/>
       <x:c r="B164" s="90"/>
       <x:c r="C164" s="90"/>
       <x:c r="D164" s="90"/>
@@ -3048,7 +3067,7 @@
       <x:c r="I164" s="102"/>
     </x:row>
     <x:row r="165">
-      <x:c r="A165" s="93"/>
+      <x:c r="A165" s="150"/>
       <x:c r="B165" s="90"/>
       <x:c r="C165" s="90"/>
       <x:c r="D165" s="90"/>
@@ -3059,7 +3078,7 @@
       <x:c r="I165" s="102"/>
     </x:row>
     <x:row r="166">
-      <x:c r="A166" s="93"/>
+      <x:c r="A166" s="150"/>
       <x:c r="B166" s="90"/>
       <x:c r="C166" s="90"/>
       <x:c r="D166" s="90"/>
@@ -3070,7 +3089,7 @@
       <x:c r="I166" s="102"/>
     </x:row>
     <x:row r="167">
-      <x:c r="A167" s="93"/>
+      <x:c r="A167" s="150"/>
       <x:c r="B167" s="90"/>
       <x:c r="C167" s="90"/>
       <x:c r="D167" s="90"/>
@@ -3081,7 +3100,7 @@
       <x:c r="I167" s="102"/>
     </x:row>
     <x:row r="168">
-      <x:c r="A168" s="93"/>
+      <x:c r="A168" s="150"/>
       <x:c r="B168" s="90"/>
       <x:c r="C168" s="90"/>
       <x:c r="D168" s="90"/>
@@ -3092,7 +3111,7 @@
       <x:c r="I168" s="102"/>
     </x:row>
     <x:row r="169">
-      <x:c r="A169" s="93"/>
+      <x:c r="A169" s="150"/>
       <x:c r="B169" s="90"/>
       <x:c r="C169" s="90"/>
       <x:c r="D169" s="90"/>
@@ -3103,7 +3122,7 @@
       <x:c r="I169" s="102"/>
     </x:row>
     <x:row r="170">
-      <x:c r="A170" s="93"/>
+      <x:c r="A170" s="150"/>
       <x:c r="B170" s="90"/>
       <x:c r="C170" s="90"/>
       <x:c r="D170" s="90"/>
@@ -3114,7 +3133,7 @@
       <x:c r="I170" s="102"/>
     </x:row>
     <x:row r="171">
-      <x:c r="A171" s="93"/>
+      <x:c r="A171" s="150"/>
       <x:c r="B171" s="90"/>
       <x:c r="C171" s="90"/>
       <x:c r="D171" s="90"/>
@@ -3125,7 +3144,7 @@
       <x:c r="I171" s="102"/>
     </x:row>
     <x:row r="172">
-      <x:c r="A172" s="93"/>
+      <x:c r="A172" s="150"/>
       <x:c r="B172" s="90"/>
       <x:c r="C172" s="90"/>
       <x:c r="D172" s="90"/>
@@ -3136,7 +3155,7 @@
       <x:c r="I172" s="102"/>
     </x:row>
     <x:row r="173">
-      <x:c r="A173" s="93"/>
+      <x:c r="A173" s="150"/>
       <x:c r="B173" s="90"/>
       <x:c r="C173" s="90"/>
       <x:c r="D173" s="90"/>
@@ -3147,7 +3166,7 @@
       <x:c r="I173" s="102"/>
     </x:row>
     <x:row r="174">
-      <x:c r="A174" s="93"/>
+      <x:c r="A174" s="150"/>
       <x:c r="B174" s="90"/>
       <x:c r="C174" s="90"/>
       <x:c r="D174" s="90"/>
@@ -3158,7 +3177,7 @@
       <x:c r="I174" s="102"/>
     </x:row>
     <x:row r="175">
-      <x:c r="A175" s="93"/>
+      <x:c r="A175" s="150"/>
       <x:c r="B175" s="90"/>
       <x:c r="C175" s="90"/>
       <x:c r="D175" s="90"/>
@@ -3169,7 +3188,7 @@
       <x:c r="I175" s="102"/>
     </x:row>
     <x:row r="176">
-      <x:c r="A176" s="93"/>
+      <x:c r="A176" s="150"/>
       <x:c r="B176" s="90"/>
       <x:c r="C176" s="90"/>
       <x:c r="D176" s="90"/>
@@ -3180,7 +3199,7 @@
       <x:c r="I176" s="102"/>
     </x:row>
     <x:row r="177">
-      <x:c r="A177" s="93"/>
+      <x:c r="A177" s="150"/>
       <x:c r="B177" s="90"/>
       <x:c r="C177" s="90"/>
       <x:c r="D177" s="90"/>
@@ -3191,7 +3210,7 @@
       <x:c r="I177" s="102"/>
     </x:row>
     <x:row r="178">
-      <x:c r="A178" s="93"/>
+      <x:c r="A178" s="150"/>
       <x:c r="B178" s="90"/>
       <x:c r="C178" s="90"/>
       <x:c r="D178" s="90"/>
@@ -3202,7 +3221,7 @@
       <x:c r="I178" s="102"/>
     </x:row>
     <x:row r="179">
-      <x:c r="A179" s="93"/>
+      <x:c r="A179" s="150"/>
       <x:c r="B179" s="90"/>
       <x:c r="C179" s="90"/>
       <x:c r="D179" s="90"/>
@@ -3213,7 +3232,7 @@
       <x:c r="I179" s="102"/>
     </x:row>
     <x:row r="180">
-      <x:c r="A180" s="93"/>
+      <x:c r="A180" s="150"/>
       <x:c r="B180" s="90"/>
       <x:c r="C180" s="90"/>
       <x:c r="D180" s="90"/>
@@ -3224,7 +3243,7 @@
       <x:c r="I180" s="102"/>
     </x:row>
     <x:row r="181">
-      <x:c r="A181" s="93"/>
+      <x:c r="A181" s="150"/>
       <x:c r="B181" s="90"/>
       <x:c r="C181" s="90"/>
       <x:c r="D181" s="90"/>
@@ -3235,7 +3254,7 @@
       <x:c r="I181" s="102"/>
     </x:row>
     <x:row r="182">
-      <x:c r="A182" s="93"/>
+      <x:c r="A182" s="150"/>
       <x:c r="B182" s="90"/>
       <x:c r="C182" s="90"/>
       <x:c r="D182" s="90"/>
@@ -3246,7 +3265,7 @@
       <x:c r="I182" s="102"/>
     </x:row>
     <x:row r="183">
-      <x:c r="A183" s="93"/>
+      <x:c r="A183" s="150"/>
       <x:c r="B183" s="90"/>
       <x:c r="C183" s="90"/>
       <x:c r="D183" s="90"/>
@@ -3257,7 +3276,7 @@
       <x:c r="I183" s="102"/>
     </x:row>
     <x:row r="184">
-      <x:c r="A184" s="93"/>
+      <x:c r="A184" s="150"/>
       <x:c r="B184" s="90"/>
       <x:c r="C184" s="90"/>
       <x:c r="D184" s="90"/>
@@ -3268,7 +3287,7 @@
       <x:c r="I184" s="102"/>
     </x:row>
     <x:row r="185">
-      <x:c r="A185" s="93"/>
+      <x:c r="A185" s="150"/>
       <x:c r="B185" s="90"/>
       <x:c r="C185" s="90"/>
       <x:c r="D185" s="90"/>
@@ -3279,7 +3298,7 @@
       <x:c r="I185" s="102"/>
     </x:row>
     <x:row r="186">
-      <x:c r="A186" s="93"/>
+      <x:c r="A186" s="150"/>
       <x:c r="B186" s="90"/>
       <x:c r="C186" s="90"/>
       <x:c r="D186" s="90"/>
@@ -3290,7 +3309,7 @@
       <x:c r="I186" s="102"/>
     </x:row>
     <x:row r="187">
-      <x:c r="A187" s="93"/>
+      <x:c r="A187" s="150"/>
       <x:c r="B187" s="90"/>
       <x:c r="C187" s="90"/>
       <x:c r="D187" s="90"/>
@@ -3301,7 +3320,7 @@
       <x:c r="I187" s="102"/>
     </x:row>
     <x:row r="188">
-      <x:c r="A188" s="93"/>
+      <x:c r="A188" s="150"/>
       <x:c r="B188" s="90"/>
       <x:c r="C188" s="90"/>
       <x:c r="D188" s="90"/>
@@ -3312,7 +3331,7 @@
       <x:c r="I188" s="102"/>
     </x:row>
     <x:row r="189">
-      <x:c r="A189" s="93"/>
+      <x:c r="A189" s="150"/>
       <x:c r="B189" s="90"/>
       <x:c r="C189" s="90"/>
       <x:c r="D189" s="90"/>
@@ -3323,7 +3342,7 @@
       <x:c r="I189" s="102"/>
     </x:row>
     <x:row r="190">
-      <x:c r="A190" s="93"/>
+      <x:c r="A190" s="150"/>
       <x:c r="B190" s="90"/>
       <x:c r="C190" s="90"/>
       <x:c r="D190" s="90"/>
@@ -3334,7 +3353,7 @@
       <x:c r="I190" s="102"/>
     </x:row>
     <x:row r="191">
-      <x:c r="A191" s="93"/>
+      <x:c r="A191" s="150"/>
       <x:c r="B191" s="90"/>
       <x:c r="C191" s="90"/>
       <x:c r="D191" s="90"/>
@@ -3345,7 +3364,7 @@
       <x:c r="I191" s="102"/>
     </x:row>
     <x:row r="192">
-      <x:c r="A192" s="93"/>
+      <x:c r="A192" s="150"/>
       <x:c r="B192" s="90"/>
       <x:c r="C192" s="90"/>
       <x:c r="D192" s="90"/>
@@ -3356,7 +3375,7 @@
       <x:c r="I192" s="102"/>
     </x:row>
     <x:row r="193">
-      <x:c r="A193" s="93"/>
+      <x:c r="A193" s="150"/>
       <x:c r="B193" s="90"/>
       <x:c r="C193" s="90"/>
       <x:c r="D193" s="90"/>
@@ -3367,7 +3386,7 @@
       <x:c r="I193" s="102"/>
     </x:row>
     <x:row r="194">
-      <x:c r="A194" s="93"/>
+      <x:c r="A194" s="150"/>
       <x:c r="B194" s="90"/>
       <x:c r="C194" s="90"/>
       <x:c r="D194" s="90"/>
@@ -3378,7 +3397,7 @@
       <x:c r="I194" s="102"/>
     </x:row>
     <x:row r="195">
-      <x:c r="A195" s="93"/>
+      <x:c r="A195" s="150"/>
       <x:c r="B195" s="90"/>
       <x:c r="C195" s="90"/>
       <x:c r="D195" s="90"/>
@@ -3389,7 +3408,7 @@
       <x:c r="I195" s="102"/>
     </x:row>
     <x:row r="196">
-      <x:c r="A196" s="93"/>
+      <x:c r="A196" s="150"/>
       <x:c r="B196" s="90"/>
       <x:c r="C196" s="90"/>
       <x:c r="D196" s="90"/>
@@ -3400,7 +3419,7 @@
       <x:c r="I196" s="102"/>
     </x:row>
     <x:row r="197">
-      <x:c r="A197" s="93"/>
+      <x:c r="A197" s="150"/>
       <x:c r="B197" s="90"/>
       <x:c r="C197" s="90"/>
       <x:c r="D197" s="90"/>
@@ -3411,7 +3430,7 @@
       <x:c r="I197" s="102"/>
     </x:row>
     <x:row r="198">
-      <x:c r="A198" s="93"/>
+      <x:c r="A198" s="150"/>
       <x:c r="B198" s="90"/>
       <x:c r="C198" s="90"/>
       <x:c r="D198" s="90"/>
@@ -3422,7 +3441,7 @@
       <x:c r="I198" s="102"/>
     </x:row>
     <x:row r="199">
-      <x:c r="A199" s="93"/>
+      <x:c r="A199" s="150"/>
       <x:c r="B199" s="90"/>
       <x:c r="C199" s="90"/>
       <x:c r="D199" s="90"/>
@@ -3433,7 +3452,7 @@
       <x:c r="I199" s="102"/>
     </x:row>
     <x:row r="200">
-      <x:c r="A200" s="94"/>
+      <x:c r="A200" s="151"/>
       <x:c r="B200" s="91"/>
       <x:c r="C200" s="91"/>
       <x:c r="D200" s="91"/>
@@ -3451,7 +3470,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b93966b7205411b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd69a48eaf6684b42"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3530,7 +3549,7 @@
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="116" t="n">
+      <x:c r="A4" s="152" t="n">
         <x:v>45663.5</x:v>
       </x:c>
       <x:c r="B4" s="117" t="str">
@@ -3560,7 +3579,7 @@
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="120" t="n">
+      <x:c r="A5" s="153" t="n">
         <x:v>45698.5</x:v>
       </x:c>
       <x:c r="B5" s="121" t="str">
@@ -3590,7 +3609,7 @@
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="120" t="n">
+      <x:c r="A6" s="153" t="n">
         <x:v>45750.5</x:v>
       </x:c>
       <x:c r="B6" s="121" t="str">
@@ -3620,7 +3639,7 @@
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="120" t="n">
+      <x:c r="A7" s="153" t="n">
         <x:v>45660.5</x:v>
       </x:c>
       <x:c r="B7" s="121" t="str">
@@ -3641,7 +3660,7 @@
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="124" t="n">
+      <x:c r="A8" s="154" t="n">
         <x:v>45810.5</x:v>
       </x:c>
       <x:c r="B8" s="125" t="str">

</xml_diff>